<commit_message>
BESP inflation adjustment, BPHEVSP adjusted to 2023 subsidy value
</commit_message>
<xml_diff>
--- a/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
+++ b/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-maryland\InputData\trans\BESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961AEFFE-5310-4A6C-8343-1D491005315D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BF71F6-A4F2-48E1-B8D0-A45B69CB7D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="59730" yWindow="2805" windowWidth="24480" windowHeight="13800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="58695" yWindow="1680" windowWidth="21825" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="285">
   <si>
     <t>BESP BAU EV Subsidy Percentage</t>
   </si>
@@ -892,6 +892,9 @@
   </si>
   <si>
     <t>which models will apply under the requirements.</t>
+  </si>
+  <si>
+    <t>Inflation adjustment (2020 to 2012 USD)</t>
   </si>
 </sst>
 </file>
@@ -905,11 +908,18 @@
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1163,38 +1173,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="38" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="38" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" pivotButton="1" applyBorder="1"/>
@@ -1210,22 +1221,23 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="6" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1236,9 +1248,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 6" xfId="1" xr:uid="{4B3EBD47-761B-4AFA-833C-3C8E79092ADC}"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -1283,7 +1297,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44965.485754629626" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44966.298819791664" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:P47" sheet="2019 Sales"/>
   </cacheSource>
@@ -2180,126 +2194,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="19">
-        <item x="10"/>
-        <item x="5"/>
-        <item x="16"/>
-        <item x="6"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="15"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="13"/>
-        <item x="11"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="17"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="14"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="19">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G22:J41" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
@@ -2419,6 +2313,126 @@
     <dataField name="Sum of JAN" fld="3" baseField="0"/>
     <dataField name="Sum of FEB" fld="4" baseField="0"/>
     <dataField name="Sum of MAR" fld="5" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="19">
+        <item x="10"/>
+        <item x="5"/>
+        <item x="16"/>
+        <item x="6"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="15"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="13"/>
+        <item x="11"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="17"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="14"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="19">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3126,7 +3140,12 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B46" s="4"/>
+      <c r="A46" s="44">
+        <v>0.88711067149387013</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>284</v>
+      </c>
       <c r="F46" s="5" t="s">
         <v>116</v>
       </c>
@@ -6411,7 +6430,7 @@
         <v>2020</v>
       </c>
       <c r="D22" s="8">
-        <f t="shared" ref="D22:I22" si="0">C22+1</f>
+        <f t="shared" ref="D22:J22" si="0">C22+1</f>
         <v>2021</v>
       </c>
       <c r="E22" s="10">
@@ -6433,6 +6452,9 @@
       <c r="I22" s="10">
         <f t="shared" si="0"/>
         <v>2026</v>
+      </c>
+      <c r="J22">
+        <v>2027</v>
       </c>
     </row>
     <row r="23" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -6441,7 +6463,7 @@
         <v>138</v>
       </c>
       <c r="C23" s="8">
-        <f t="shared" ref="C23:I24" si="1">SUMIFS(C$41:C$54,$A$41:$A$54,$C$21,$B$41:$B$54,$B23)</f>
+        <f t="shared" ref="C23:J24" si="1">SUMIFS(C$41:C$54,$A$41:$A$54,$C$21,$B$41:$B$54,$B23)</f>
         <v>2500</v>
       </c>
       <c r="D23" s="10">
@@ -6454,19 +6476,23 @@
       </c>
       <c r="F23" s="10">
         <f t="shared" si="1"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="G23" s="10">
         <f t="shared" si="1"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H23" s="10">
         <f t="shared" si="1"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="I23" s="10">
         <f t="shared" si="1"/>
-        <v>2500</v>
+        <v>3000</v>
+      </c>
+      <c r="J23" s="10">
+        <f t="shared" si="1"/>
+        <v>3000</v>
       </c>
     </row>
     <row r="24" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -6502,8 +6528,45 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="J24" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C25">
+        <f>C23*About!$A46</f>
+        <v>2217.7766787346754</v>
+      </c>
+      <c r="D25">
+        <f>D23*About!$A46</f>
+        <v>2217.7766787346754</v>
+      </c>
+      <c r="E25">
+        <f>E23*About!$A46</f>
+        <v>2217.7766787346754</v>
+      </c>
+      <c r="F25">
+        <f>F23*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="G25">
+        <f>G23*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="H25">
+        <f>H23*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="I25">
+        <f>I23*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="J25">
+        <f>J23*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+    </row>
     <row r="26" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31"/>
       <c r="B26" s="31"/>
@@ -6964,11 +7027,11 @@
         <v>5245.8606136031603</v>
       </c>
       <c r="B33" s="12">
-        <f t="shared" ref="B33:AF33" si="2">(B3+D23)</f>
+        <f>(B3+C23)</f>
         <v>5245.8606136031594</v>
       </c>
       <c r="C33" s="12">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="C33:AF33" si="2">(C3+D23)</f>
         <v>5245.8606136031603</v>
       </c>
       <c r="D33" s="12">
@@ -6977,23 +7040,23 @@
       </c>
       <c r="E33" s="12">
         <f t="shared" si="2"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="F33" s="12">
         <f t="shared" si="2"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="G33" s="12">
         <f t="shared" si="2"/>
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="J33" s="12">
         <f t="shared" si="2"/>
@@ -7582,16 +7645,19 @@
         <v>2500</v>
       </c>
       <c r="F50" s="10">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="G50" s="10">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H50" s="10">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="I50" s="10">
-        <v>2500</v>
+        <v>3000</v>
+      </c>
+      <c r="J50" s="56">
+        <v>3000</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -11247,13 +11313,13 @@
       <c r="G24" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="H24" s="46">
+      <c r="H24" s="47">
         <v>175</v>
       </c>
-      <c r="I24" s="47">
+      <c r="I24" s="48">
         <v>210</v>
       </c>
-      <c r="J24" s="48">
+      <c r="J24" s="49">
         <v>45</v>
       </c>
       <c r="K24" s="8">
@@ -11271,13 +11337,13 @@
       <c r="G25" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="49">
+      <c r="H25" s="50">
         <v>997</v>
       </c>
-      <c r="I25" s="50">
+      <c r="I25" s="51">
         <v>1111</v>
       </c>
-      <c r="J25" s="51">
+      <c r="J25" s="52">
         <v>1147</v>
       </c>
       <c r="K25" s="8">
@@ -11295,13 +11361,13 @@
       <c r="G26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="H26" s="49">
+      <c r="H26" s="50">
         <v>72</v>
       </c>
-      <c r="I26" s="50">
+      <c r="I26" s="51">
         <v>87</v>
       </c>
-      <c r="J26" s="51">
+      <c r="J26" s="52">
         <v>33</v>
       </c>
       <c r="K26" s="8">
@@ -11319,13 +11385,13 @@
       <c r="G27" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="49">
+      <c r="H27" s="50">
         <v>557</v>
       </c>
-      <c r="I27" s="50">
+      <c r="I27" s="51">
         <v>573</v>
       </c>
-      <c r="J27" s="51">
+      <c r="J27" s="52">
         <v>611</v>
       </c>
       <c r="K27" s="8">
@@ -11343,13 +11409,13 @@
       <c r="G28" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H28" s="49">
+      <c r="H28" s="50">
         <v>2044</v>
       </c>
-      <c r="I28" s="50">
+      <c r="I28" s="51">
         <v>2430</v>
       </c>
-      <c r="J28" s="51">
+      <c r="J28" s="52">
         <v>3782</v>
       </c>
       <c r="K28" s="8">
@@ -11367,13 +11433,13 @@
       <c r="G29" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="H29" s="49">
+      <c r="H29" s="50">
         <v>1270</v>
       </c>
-      <c r="I29" s="50">
+      <c r="I29" s="51">
         <v>1281</v>
       </c>
-      <c r="J29" s="51">
+      <c r="J29" s="52">
         <v>1403</v>
       </c>
       <c r="K29" s="8">
@@ -11391,13 +11457,13 @@
       <c r="G30" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="H30" s="49">
+      <c r="H30" s="50">
         <v>111</v>
       </c>
-      <c r="I30" s="50">
+      <c r="I30" s="51">
         <v>173</v>
       </c>
-      <c r="J30" s="51">
+      <c r="J30" s="52">
         <v>256</v>
       </c>
       <c r="K30" s="8">
@@ -11415,13 +11481,13 @@
       <c r="G31" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="H31" s="49">
+      <c r="H31" s="50">
         <v>210</v>
       </c>
-      <c r="I31" s="50">
+      <c r="I31" s="51">
         <v>186</v>
       </c>
-      <c r="J31" s="51">
+      <c r="J31" s="52">
         <v>212</v>
       </c>
       <c r="K31" s="8">
@@ -11439,13 +11505,13 @@
       <c r="G32" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="H32" s="49">
+      <c r="H32" s="50">
         <v>309</v>
       </c>
-      <c r="I32" s="50">
+      <c r="I32" s="51">
         <v>517</v>
       </c>
-      <c r="J32" s="51">
+      <c r="J32" s="52">
         <v>240</v>
       </c>
       <c r="K32" s="8">
@@ -11463,13 +11529,13 @@
       <c r="G33" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="H33" s="49">
+      <c r="H33" s="50">
         <v>398</v>
       </c>
-      <c r="I33" s="50">
+      <c r="I33" s="51">
         <v>382</v>
       </c>
-      <c r="J33" s="51">
+      <c r="J33" s="52">
         <v>532</v>
       </c>
       <c r="K33" s="8">
@@ -11487,13 +11553,13 @@
       <c r="G34" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="49">
+      <c r="H34" s="50">
         <v>133</v>
       </c>
-      <c r="I34" s="50">
+      <c r="I34" s="51">
         <v>157</v>
       </c>
-      <c r="J34" s="51">
+      <c r="J34" s="52">
         <v>341</v>
       </c>
       <c r="K34" s="8">
@@ -11511,13 +11577,13 @@
       <c r="G35" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="H35" s="49">
+      <c r="H35" s="50">
         <v>717</v>
       </c>
-      <c r="I35" s="50">
+      <c r="I35" s="51">
         <v>654</v>
       </c>
-      <c r="J35" s="51">
+      <c r="J35" s="52">
         <v>1314</v>
       </c>
       <c r="K35" s="8">
@@ -11535,13 +11601,13 @@
       <c r="G36" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="H36" s="49">
+      <c r="H36" s="50">
         <v>215</v>
       </c>
-      <c r="I36" s="50">
+      <c r="I36" s="51">
         <v>255</v>
       </c>
-      <c r="J36" s="51">
+      <c r="J36" s="52">
         <v>310</v>
       </c>
       <c r="K36" s="8">
@@ -11559,11 +11625,11 @@
       <c r="G37" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="49"/>
-      <c r="I37" s="50">
+      <c r="H37" s="50"/>
+      <c r="I37" s="51">
         <v>27</v>
       </c>
-      <c r="J37" s="51">
+      <c r="J37" s="52">
         <v>52</v>
       </c>
       <c r="K37" s="8">
@@ -11581,13 +11647,13 @@
       <c r="G38" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="H38" s="49">
+      <c r="H38" s="50">
         <v>8000</v>
       </c>
-      <c r="I38" s="50">
+      <c r="I38" s="51">
         <v>7275</v>
       </c>
-      <c r="J38" s="51">
+      <c r="J38" s="52">
         <v>14625</v>
       </c>
       <c r="K38" s="8">
@@ -11605,13 +11671,13 @@
       <c r="G39" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="H39" s="49">
+      <c r="H39" s="50">
         <v>1123</v>
       </c>
-      <c r="I39" s="50">
+      <c r="I39" s="51">
         <v>1205</v>
       </c>
-      <c r="J39" s="51">
+      <c r="J39" s="52">
         <v>1820</v>
       </c>
       <c r="K39" s="8">
@@ -11629,13 +11695,13 @@
       <c r="G40" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="H40" s="49">
+      <c r="H40" s="50">
         <v>220</v>
       </c>
-      <c r="I40" s="50">
+      <c r="I40" s="51">
         <v>250</v>
       </c>
-      <c r="J40" s="51">
+      <c r="J40" s="52">
         <v>335</v>
       </c>
       <c r="K40" s="8">
@@ -11653,13 +11719,13 @@
       <c r="G41" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="H41" s="52">
+      <c r="H41" s="53">
         <v>164</v>
       </c>
-      <c r="I41" s="53">
+      <c r="I41" s="54">
         <v>118</v>
       </c>
-      <c r="J41" s="54">
+      <c r="J41" s="55">
         <v>581</v>
       </c>
       <c r="K41" s="8">
@@ -20383,7 +20449,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>262</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -20397,7 +20463,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="45"/>
+      <c r="A2" s="46"/>
       <c r="B2" s="8" t="s">
         <v>266</v>
       </c>
@@ -20409,7 +20475,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="45"/>
+      <c r="A3" s="46"/>
       <c r="C3" s="8">
         <v>200000</v>
       </c>
@@ -20418,7 +20484,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="45"/>
+      <c r="A4" s="46"/>
       <c r="D4" s="8">
         <v>200000</v>
       </c>
@@ -21777,142 +21843,142 @@
       </c>
       <c r="B2" s="38">
         <f>C2</f>
-        <v>5245.8606136031603</v>
+        <v>4653.658931496745</v>
       </c>
       <c r="C2" s="38">
         <f>D2</f>
-        <v>5245.8606136031603</v>
+        <v>4653.658931496745</v>
       </c>
       <c r="D2" s="38">
         <f>E2</f>
-        <v>5245.8606136031603</v>
+        <v>4653.658931496745</v>
       </c>
       <c r="E2" s="39">
-        <f>Data!A33</f>
-        <v>5245.8606136031603</v>
-      </c>
-      <c r="F2" s="39">
-        <f>Data!B33</f>
-        <v>5245.8606136031594</v>
-      </c>
-      <c r="G2" s="39">
-        <f>Data!C33</f>
-        <v>5245.8606136031603</v>
-      </c>
-      <c r="H2" s="39">
-        <f>Data!D33</f>
-        <v>4413.0458308533107</v>
-      </c>
-      <c r="I2" s="39">
-        <f>Data!E33</f>
-        <v>2500</v>
-      </c>
-      <c r="J2" s="39">
-        <f>Data!F33</f>
-        <v>2500</v>
-      </c>
-      <c r="K2" s="39">
-        <f>Data!G33</f>
-        <v>2500</v>
-      </c>
-      <c r="L2" s="39">
-        <f>Data!H33</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="39">
-        <f>Data!I33</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="39">
-        <f>Data!J33</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="39">
-        <f>Data!K33</f>
-        <v>0</v>
-      </c>
-      <c r="P2" s="39">
-        <f>Data!L33</f>
-        <v>0</v>
-      </c>
-      <c r="Q2" s="39">
-        <f>Data!M33</f>
-        <v>0</v>
-      </c>
-      <c r="R2" s="39">
-        <f>Data!N33</f>
-        <v>0</v>
-      </c>
-      <c r="S2" s="39">
-        <f>Data!O33</f>
-        <v>0</v>
-      </c>
-      <c r="T2" s="39">
-        <f>Data!P33</f>
-        <v>0</v>
-      </c>
-      <c r="U2" s="39">
-        <f>Data!Q33</f>
-        <v>0</v>
-      </c>
-      <c r="V2" s="39">
-        <f>Data!R33</f>
-        <v>0</v>
-      </c>
-      <c r="W2" s="39">
-        <f>Data!S33</f>
-        <v>0</v>
-      </c>
-      <c r="X2" s="39">
-        <f>Data!T33</f>
-        <v>0</v>
-      </c>
-      <c r="Y2" s="39">
-        <f>Data!U33</f>
-        <v>0</v>
-      </c>
-      <c r="Z2" s="39">
-        <f>Data!V33</f>
-        <v>0</v>
-      </c>
-      <c r="AA2" s="39">
-        <f>Data!W33</f>
-        <v>0</v>
-      </c>
-      <c r="AB2" s="39">
-        <f>Data!X33</f>
-        <v>0</v>
-      </c>
-      <c r="AC2" s="39">
-        <f>Data!Y33</f>
-        <v>0</v>
-      </c>
-      <c r="AD2" s="39">
-        <f>Data!Z33</f>
-        <v>0</v>
-      </c>
-      <c r="AE2" s="39">
-        <f>Data!AA33</f>
-        <v>0</v>
-      </c>
-      <c r="AF2" s="39">
-        <f>Data!AB33</f>
-        <v>0</v>
-      </c>
-      <c r="AG2" s="39">
-        <f>Data!AC33</f>
-        <v>0</v>
-      </c>
-      <c r="AH2" s="39">
-        <f>Data!AD33</f>
-        <v>0</v>
-      </c>
-      <c r="AI2" s="39">
-        <f>Data!AE33</f>
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="39">
-        <f>Data!AF33</f>
+        <f>Data!A33*About!$A46</f>
+        <v>4653.658931496745</v>
+      </c>
+      <c r="F2" s="12">
+        <f>Data!B33*About!$A46</f>
+        <v>4653.6589314967441</v>
+      </c>
+      <c r="G2" s="12">
+        <f>Data!C33*About!$A46</f>
+        <v>4653.658931496745</v>
+      </c>
+      <c r="H2" s="12">
+        <f>Data!D33*About!$A46</f>
+        <v>3914.8600503415046</v>
+      </c>
+      <c r="I2" s="12">
+        <f>Data!E33*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="J2" s="12">
+        <f>Data!F33*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="K2" s="12">
+        <f>Data!G33*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="L2" s="12">
+        <f>Data!H33*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="M2" s="12">
+        <f>Data!I33*About!$A46</f>
+        <v>2661.3320144816103</v>
+      </c>
+      <c r="N2" s="12">
+        <f>Data!J33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="12">
+        <f>Data!K33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="P2" s="12">
+        <f>Data!L33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="12">
+        <f>Data!M33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="12">
+        <f>Data!N33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="S2" s="12">
+        <f>Data!O33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="T2" s="12">
+        <f>Data!P33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="U2" s="12">
+        <f>Data!Q33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="V2" s="12">
+        <f>Data!R33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="W2" s="12">
+        <f>Data!S33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="X2" s="12">
+        <f>Data!T33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="12">
+        <f>Data!U33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="12">
+        <f>Data!V33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AA2" s="12">
+        <f>Data!W33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AB2" s="12">
+        <f>Data!X33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AC2" s="12">
+        <f>Data!Y33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AD2" s="12">
+        <f>Data!Z33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AE2" s="12">
+        <f>Data!AA33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AF2" s="12">
+        <f>Data!AB33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AG2" s="12">
+        <f>Data!AC33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AH2" s="12">
+        <f>Data!AD33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AI2" s="12">
+        <f>Data!AE33*About!$A46</f>
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="12">
+        <f>Data!AF33*About!$A46</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates to ICCT input data to account for entities of concern requirement
</commit_message>
<xml_diff>
--- a/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
+++ b/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-maryland\InputData\trans\BESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BF71F6-A4F2-48E1-B8D0-A45B69CB7D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F06C96E-F650-40AA-AB4E-417D6B5DAC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58695" yWindow="1680" windowWidth="21825" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="61320" yWindow="1935" windowWidth="23100" windowHeight="13305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId8"/>
+    <pivotCache cacheId="11" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1177,7 +1177,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1248,7 +1248,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1297,7 +1296,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44966.298819791664" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44993.366300347225" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:P47" sheet="2019 Sales"/>
   </cacheSource>
@@ -2194,7 +2193,127 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="19">
+        <item x="10"/>
+        <item x="5"/>
+        <item x="16"/>
+        <item x="6"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="15"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="13"/>
+        <item x="11"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="17"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="14"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="19">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G22:J41" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
@@ -2313,126 +2432,6 @@
     <dataField name="Sum of JAN" fld="3" baseField="0"/>
     <dataField name="Sum of FEB" fld="4" baseField="0"/>
     <dataField name="Sum of MAR" fld="5" baseField="0"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="19">
-        <item x="10"/>
-        <item x="5"/>
-        <item x="16"/>
-        <item x="6"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="15"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="13"/>
-        <item x="11"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="17"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="14"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="19">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -6188,72 +6187,95 @@
         <v>1913.0458308533109</v>
       </c>
       <c r="E3" s="11">
-        <v>0</v>
+        <f>BAU!G92</f>
+        <v>1531.9111519939402</v>
       </c>
       <c r="F3" s="11">
-        <v>0</v>
+        <f>BAU!H92</f>
+        <v>1131.4322818029341</v>
       </c>
       <c r="G3" s="11">
-        <v>0</v>
+        <f>BAU!I92</f>
+        <v>933.18813916995919</v>
       </c>
       <c r="H3" s="11">
-        <v>0</v>
+        <f>BAU!J92</f>
+        <v>933.18813916995953</v>
       </c>
       <c r="I3" s="11">
-        <v>0</v>
+        <f>BAU!K92</f>
+        <v>744.00735890914916</v>
       </c>
       <c r="J3" s="11">
-        <v>0</v>
+        <f>BAU!L92</f>
+        <v>744.00735890914984</v>
       </c>
       <c r="K3" s="11">
-        <v>0</v>
+        <f>BAU!M92</f>
+        <v>621.92251501542137</v>
       </c>
       <c r="L3" s="11">
-        <v>0</v>
+        <f>BAU!N92</f>
+        <v>240.24673989502756</v>
       </c>
       <c r="M3" s="11">
-        <v>0</v>
+        <f>BAU!O92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="N3" s="11">
-        <v>0</v>
+        <f>BAU!P92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="O3" s="11">
-        <v>0</v>
+        <f>BAU!Q92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="P3" s="11">
-        <v>0</v>
+        <f>BAU!R92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q3" s="11">
-        <v>0</v>
+        <f>BAU!S92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="R3" s="11">
-        <v>0</v>
+        <f>BAU!T92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="S3" s="11">
-        <v>0</v>
+        <f>BAU!U92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="T3" s="11">
+        <f>BAU!V92</f>
         <v>0</v>
       </c>
       <c r="U3" s="11">
+        <f>BAU!W92</f>
         <v>0</v>
       </c>
       <c r="V3" s="11">
+        <f>BAU!X92</f>
         <v>0</v>
       </c>
       <c r="W3" s="11">
+        <f>BAU!Y92</f>
         <v>0</v>
       </c>
       <c r="X3" s="11">
+        <f>BAU!Z92</f>
         <v>0</v>
       </c>
       <c r="Y3" s="11">
+        <f>BAU!AA92</f>
         <v>0</v>
       </c>
       <c r="Z3" s="11">
+        <f>BAU!AB92</f>
         <v>0</v>
       </c>
       <c r="AA3" s="11">
+        <f>BAU!AC92</f>
         <v>0</v>
       </c>
       <c r="AB3" s="11">
@@ -6430,7 +6452,7 @@
         <v>2020</v>
       </c>
       <c r="D22" s="8">
-        <f t="shared" ref="D22:J22" si="0">C22+1</f>
+        <f t="shared" ref="D22:I22" si="0">C22+1</f>
         <v>2021</v>
       </c>
       <c r="E22" s="10">
@@ -7040,63 +7062,63 @@
       </c>
       <c r="E33" s="12">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>4531.9111519939397</v>
       </c>
       <c r="F33" s="12">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>4131.4322818029341</v>
       </c>
       <c r="G33" s="12">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>3933.188139169959</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>3933.1881391699594</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>3744.0073589091489</v>
       </c>
       <c r="J33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>744.00735890914984</v>
       </c>
       <c r="K33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>621.92251501542137</v>
       </c>
       <c r="L33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>240.24673989502756</v>
       </c>
       <c r="M33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="N33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="O33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="P33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="R33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="S33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="T33" s="12">
         <f t="shared" si="2"/>
@@ -7656,7 +7678,7 @@
       <c r="I50" s="10">
         <v>3000</v>
       </c>
-      <c r="J50" s="56">
+      <c r="J50" s="43">
         <v>3000</v>
       </c>
     </row>
@@ -21871,63 +21893,63 @@
       </c>
       <c r="I2" s="12">
         <f>Data!E33*About!$A46</f>
-        <v>2661.3320144816103</v>
+        <v>4020.3067451959023</v>
       </c>
       <c r="J2" s="12">
         <f>Data!F33*About!$A46</f>
-        <v>2661.3320144816103</v>
+        <v>3665.0376657416527</v>
       </c>
       <c r="K2" s="12">
         <f>Data!G33*About!$A46</f>
-        <v>2661.3320144816103</v>
+        <v>3489.1731712507876</v>
       </c>
       <c r="L2" s="12">
         <f>Data!H33*About!$A46</f>
-        <v>2661.3320144816103</v>
+        <v>3489.1731712507881</v>
       </c>
       <c r="M2" s="12">
         <f>Data!I33*About!$A46</f>
-        <v>2661.3320144816103</v>
+        <v>3321.3488822398863</v>
       </c>
       <c r="N2" s="12">
         <f>Data!J33*About!$A46</f>
-        <v>0</v>
+        <v>660.0168677582767</v>
       </c>
       <c r="O2" s="12">
         <f>Data!K33*About!$A46</f>
-        <v>0</v>
+        <v>551.71409991248697</v>
       </c>
       <c r="P2" s="12">
         <f>Data!L33*About!$A46</f>
-        <v>0</v>
+        <v>213.12544675249106</v>
       </c>
       <c r="Q2" s="12">
         <f>Data!M33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="R2" s="12">
         <f>Data!N33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="S2" s="12">
         <f>Data!O33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="T2" s="12">
         <f>Data!P33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="U2" s="12">
         <f>Data!Q33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="V2" s="12">
         <f>Data!R33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="W2" s="12">
         <f>Data!S33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="X2" s="12">
         <f>Data!T33*About!$A46</f>

</xml_diff>